<commit_message>
Le Régent : identifiants produits uniques (rg_) pour éviter de reprendre photos/réglages d'autres cartes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SbCGX2wzJDQPrwbkenBcxS
</commit_message>
<xml_diff>
--- a/cartes/Carte_Le_Regent.xlsx
+++ b/cartes/Carte_Le_Regent.xlsx
@@ -653,7 +653,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ca1</t>
+          <t>rg_ca1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -691,7 +691,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ca2</t>
+          <t>rg_ca2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -729,7 +729,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ca3</t>
+          <t>rg_ca3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ca4</t>
+          <t>rg_ca4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -915,7 +915,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>dg1</t>
+          <t>rg_dg1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -958,7 +958,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>dg2</t>
+          <t>rg_dg2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2872,7 +2872,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>pl1</t>
+          <t>rg_pl1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pl3</t>
+          <t>rg_pl3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2922,7 +2922,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>pl8</t>
+          <t>rg_pl8</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2947,7 +2947,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>pl9</t>
+          <t>rg_pl9</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2972,7 +2972,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pl10</t>
+          <t>rg_pl10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2997,7 +2997,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>enf1</t>
+          <t>rg_enf1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3022,7 +3022,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>enf1</t>
+          <t>rg_enf1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>d2</t>
+          <t>rg_d2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3072,7 +3072,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>d3</t>
+          <t>rg_d3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3097,7 +3097,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>rg_d12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3122,7 +3122,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>d4</t>
+          <t>rg_d4</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3147,7 +3147,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>d5</t>
+          <t>rg_d5</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3172,7 +3172,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>d6</t>
+          <t>rg_d6</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>d9</t>
+          <t>rg_d9</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3222,7 +3222,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>rg_d12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3247,7 +3247,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>d2</t>
+          <t>rg_d2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3272,7 +3272,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>d4</t>
+          <t>rg_d4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3297,7 +3297,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>d5</t>
+          <t>rg_d5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3322,7 +3322,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>d6</t>
+          <t>rg_d6</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>d7</t>
+          <t>rg_d7</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3372,7 +3372,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>d8</t>
+          <t>rg_d8</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3397,7 +3397,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>d9</t>
+          <t>rg_d9</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3422,7 +3422,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>rg_d10</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3447,7 +3447,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>rg_d13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3472,7 +3472,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>rg_d14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ap8</t>
+          <t>rg_ap8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3522,7 +3522,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ap9</t>
+          <t>rg_ap9</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3547,7 +3547,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>so1</t>
+          <t>rg_so1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3572,7 +3572,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>so2</t>
+          <t>rg_so2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3597,7 +3597,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>so4</t>
+          <t>rg_so4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3622,7 +3622,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>so5</t>
+          <t>rg_so5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>so6</t>
+          <t>rg_so6</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3672,7 +3672,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>so7</t>
+          <t>rg_so7</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3697,7 +3697,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ca1</t>
+          <t>rg_ca1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3722,7 +3722,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ca2</t>
+          <t>rg_ca2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3747,7 +3747,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ca3</t>
+          <t>rg_ca3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3772,7 +3772,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>dg1</t>
+          <t>rg_dg1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>dg2</t>
+          <t>rg_dg2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3822,7 +3822,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>vi3</t>
+          <t>rg_vi3</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3847,7 +3847,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>vi4</t>
+          <t>rg_vi4</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3872,7 +3872,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>vi5</t>
+          <t>rg_vi5</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3897,7 +3897,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>vi6</t>
+          <t>rg_vi6</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3922,7 +3922,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>vi7</t>
+          <t>rg_vi7</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>vi8</t>
+          <t>rg_vi8</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gr1</t>
+          <t>rg_gr1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4325,7 +4325,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>gr2</t>
+          <t>rg_gr2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4368,7 +4368,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>gr3</t>
+          <t>rg_gr3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4411,7 +4411,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>gr4</t>
+          <t>rg_gr4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4564,7 +4564,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>pl1</t>
+          <t>rg_pl1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4612,7 +4612,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pl2</t>
+          <t>rg_pl2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4660,7 +4660,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>pl3</t>
+          <t>rg_pl3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4708,7 +4708,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>pl4</t>
+          <t>rg_pl4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4756,7 +4756,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pl5</t>
+          <t>rg_pl5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4804,7 +4804,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>pl6</t>
+          <t>rg_pl6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4852,7 +4852,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>pl7</t>
+          <t>rg_pl7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4900,7 +4900,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>pl8</t>
+          <t>rg_pl8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4948,7 +4948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>pl9</t>
+          <t>rg_pl9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4996,7 +4996,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>pl10</t>
+          <t>rg_pl10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5044,7 +5044,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>pl11</t>
+          <t>rg_pl11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5092,7 +5092,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>pl12</t>
+          <t>rg_pl12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -5135,7 +5135,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>pl13</t>
+          <t>rg_pl13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5288,7 +5288,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>enf1</t>
+          <t>rg_enf1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5441,7 +5441,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>d1</t>
+          <t>rg_d1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5484,7 +5484,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>d2</t>
+          <t>rg_d2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5532,7 +5532,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>d3</t>
+          <t>rg_d3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5580,7 +5580,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>d4</t>
+          <t>rg_d4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -5623,7 +5623,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>d5</t>
+          <t>rg_d5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5666,7 +5666,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>d6</t>
+          <t>rg_d6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5709,7 +5709,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>d7</t>
+          <t>rg_d7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5752,7 +5752,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>d8</t>
+          <t>rg_d8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5795,7 +5795,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>d9</t>
+          <t>rg_d9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -5838,7 +5838,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>rg_d10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5881,7 +5881,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>rg_d11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5929,7 +5929,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>rg_d12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -5977,7 +5977,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>rg_d13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6025,7 +6025,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>rg_d14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6183,7 +6183,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ap1</t>
+          <t>rg_ap1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6231,7 +6231,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ap2</t>
+          <t>rg_ap2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6279,7 +6279,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ap3</t>
+          <t>rg_ap3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6327,7 +6327,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ap4</t>
+          <t>rg_ap4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6375,7 +6375,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ap5</t>
+          <t>rg_ap5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6423,7 +6423,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ap6</t>
+          <t>rg_ap6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6471,7 +6471,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ap7</t>
+          <t>rg_ap7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6519,7 +6519,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ap8</t>
+          <t>rg_ap8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6567,7 +6567,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ap9</t>
+          <t>rg_ap9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6615,7 +6615,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ap10</t>
+          <t>rg_ap10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6663,7 +6663,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ap11</t>
+          <t>rg_ap11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6711,7 +6711,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ap12</t>
+          <t>rg_ap12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6759,7 +6759,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ap13</t>
+          <t>rg_ap13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>vi1</t>
+          <t>rg_vi1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6965,7 +6965,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>vi2</t>
+          <t>rg_vi2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -7013,7 +7013,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>vi3</t>
+          <t>rg_vi3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -7061,7 +7061,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>vi4</t>
+          <t>rg_vi4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -7109,7 +7109,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>vi5</t>
+          <t>rg_vi5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>vi6</t>
+          <t>rg_vi6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7205,7 +7205,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>vi7</t>
+          <t>rg_vi7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -7253,7 +7253,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>vi8</t>
+          <t>rg_vi8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7301,7 +7301,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>vi9</t>
+          <t>rg_vi9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7349,7 +7349,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>vi10</t>
+          <t>rg_vi10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>vi11</t>
+          <t>rg_vi11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7445,7 +7445,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>vi12</t>
+          <t>rg_vi12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7493,7 +7493,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>vi13</t>
+          <t>rg_vi13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7651,7 +7651,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>so1</t>
+          <t>rg_so1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -7699,7 +7699,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>so2</t>
+          <t>rg_so2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -7747,7 +7747,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>so3</t>
+          <t>rg_so3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -7795,7 +7795,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>so4</t>
+          <t>rg_so4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -7843,7 +7843,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>so5</t>
+          <t>rg_so5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7891,7 +7891,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>so6</t>
+          <t>rg_so6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7939,7 +7939,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>so7</t>
+          <t>rg_so7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">

</xml_diff>

<commit_message>
Le Régent : préfixe re_ (règle 2 lettres du nom du restaurant)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SbCGX2wzJDQPrwbkenBcxS
</commit_message>
<xml_diff>
--- a/cartes/Carte_Le_Regent.xlsx
+++ b/cartes/Carte_Le_Regent.xlsx
@@ -653,7 +653,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rg_ca1</t>
+          <t>re_ca1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -691,7 +691,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rg_ca2</t>
+          <t>re_ca2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -729,7 +729,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rg_ca3</t>
+          <t>re_ca3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rg_ca4</t>
+          <t>re_ca4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -915,7 +915,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rg_dg1</t>
+          <t>re_dg1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -958,7 +958,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rg_dg2</t>
+          <t>re_dg2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2872,7 +2872,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rg_pl1</t>
+          <t>re_pl1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rg_pl3</t>
+          <t>re_pl3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2922,7 +2922,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rg_pl8</t>
+          <t>re_pl8</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2947,7 +2947,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rg_pl9</t>
+          <t>re_pl9</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2972,7 +2972,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rg_pl10</t>
+          <t>re_pl10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2997,7 +2997,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rg_enf1</t>
+          <t>re_enf1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3022,7 +3022,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rg_enf1</t>
+          <t>re_enf1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>rg_d2</t>
+          <t>re_d2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3072,7 +3072,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>rg_d3</t>
+          <t>re_d3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3097,7 +3097,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>rg_d12</t>
+          <t>re_d12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3122,7 +3122,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>rg_d4</t>
+          <t>re_d4</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3147,7 +3147,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rg_d5</t>
+          <t>re_d5</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3172,7 +3172,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>rg_d6</t>
+          <t>re_d6</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>rg_d9</t>
+          <t>re_d9</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3222,7 +3222,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>rg_d12</t>
+          <t>re_d12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3247,7 +3247,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>rg_d2</t>
+          <t>re_d2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3272,7 +3272,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>rg_d4</t>
+          <t>re_d4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3297,7 +3297,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>rg_d5</t>
+          <t>re_d5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3322,7 +3322,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>rg_d6</t>
+          <t>re_d6</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>rg_d7</t>
+          <t>re_d7</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3372,7 +3372,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>rg_d8</t>
+          <t>re_d8</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3397,7 +3397,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>rg_d9</t>
+          <t>re_d9</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3422,7 +3422,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>rg_d10</t>
+          <t>re_d10</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3447,7 +3447,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>rg_d13</t>
+          <t>re_d13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3472,7 +3472,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>rg_d14</t>
+          <t>re_d14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>rg_ap8</t>
+          <t>re_ap8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3522,7 +3522,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>rg_ap9</t>
+          <t>re_ap9</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3547,7 +3547,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>rg_so1</t>
+          <t>re_so1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3572,7 +3572,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>rg_so2</t>
+          <t>re_so2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3597,7 +3597,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>rg_so4</t>
+          <t>re_so4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3622,7 +3622,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>rg_so5</t>
+          <t>re_so5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>rg_so6</t>
+          <t>re_so6</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3672,7 +3672,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>rg_so7</t>
+          <t>re_so7</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3697,7 +3697,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>rg_ca1</t>
+          <t>re_ca1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3722,7 +3722,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>rg_ca2</t>
+          <t>re_ca2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3747,7 +3747,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>rg_ca3</t>
+          <t>re_ca3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3772,7 +3772,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>rg_dg1</t>
+          <t>re_dg1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>rg_dg2</t>
+          <t>re_dg2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3822,7 +3822,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>rg_vi3</t>
+          <t>re_vi3</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3847,7 +3847,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>rg_vi4</t>
+          <t>re_vi4</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3872,7 +3872,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>rg_vi5</t>
+          <t>re_vi5</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3897,7 +3897,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>rg_vi6</t>
+          <t>re_vi6</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3922,7 +3922,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>rg_vi7</t>
+          <t>re_vi7</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>rg_vi8</t>
+          <t>re_vi8</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rg_gr1</t>
+          <t>re_gr1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4325,7 +4325,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rg_gr2</t>
+          <t>re_gr2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4368,7 +4368,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rg_gr3</t>
+          <t>re_gr3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4411,7 +4411,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rg_gr4</t>
+          <t>re_gr4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4564,7 +4564,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rg_pl1</t>
+          <t>re_pl1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4612,7 +4612,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rg_pl2</t>
+          <t>re_pl2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4660,7 +4660,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rg_pl3</t>
+          <t>re_pl3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4708,7 +4708,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rg_pl4</t>
+          <t>re_pl4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4756,7 +4756,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rg_pl5</t>
+          <t>re_pl5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4804,7 +4804,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rg_pl6</t>
+          <t>re_pl6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4852,7 +4852,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rg_pl7</t>
+          <t>re_pl7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4900,7 +4900,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>rg_pl8</t>
+          <t>re_pl8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4948,7 +4948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>rg_pl9</t>
+          <t>re_pl9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4996,7 +4996,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>rg_pl10</t>
+          <t>re_pl10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5044,7 +5044,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>rg_pl11</t>
+          <t>re_pl11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5092,7 +5092,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rg_pl12</t>
+          <t>re_pl12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -5135,7 +5135,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>rg_pl13</t>
+          <t>re_pl13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5288,7 +5288,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rg_enf1</t>
+          <t>re_enf1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5441,7 +5441,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rg_d1</t>
+          <t>re_d1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5484,7 +5484,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rg_d2</t>
+          <t>re_d2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5532,7 +5532,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rg_d3</t>
+          <t>re_d3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5580,7 +5580,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rg_d4</t>
+          <t>re_d4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -5623,7 +5623,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rg_d5</t>
+          <t>re_d5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5666,7 +5666,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rg_d6</t>
+          <t>re_d6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5709,7 +5709,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rg_d7</t>
+          <t>re_d7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5752,7 +5752,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>rg_d8</t>
+          <t>re_d8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5795,7 +5795,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>rg_d9</t>
+          <t>re_d9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -5838,7 +5838,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>rg_d10</t>
+          <t>re_d10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5881,7 +5881,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>rg_d11</t>
+          <t>re_d11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5929,7 +5929,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rg_d12</t>
+          <t>re_d12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -5977,7 +5977,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>rg_d13</t>
+          <t>re_d13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6025,7 +6025,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>rg_d14</t>
+          <t>re_d14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6183,7 +6183,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rg_ap1</t>
+          <t>re_ap1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6231,7 +6231,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rg_ap2</t>
+          <t>re_ap2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6279,7 +6279,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rg_ap3</t>
+          <t>re_ap3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6327,7 +6327,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rg_ap4</t>
+          <t>re_ap4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6375,7 +6375,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rg_ap5</t>
+          <t>re_ap5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6423,7 +6423,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rg_ap6</t>
+          <t>re_ap6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6471,7 +6471,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rg_ap7</t>
+          <t>re_ap7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6519,7 +6519,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>rg_ap8</t>
+          <t>re_ap8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6567,7 +6567,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>rg_ap9</t>
+          <t>re_ap9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6615,7 +6615,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>rg_ap10</t>
+          <t>re_ap10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6663,7 +6663,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>rg_ap11</t>
+          <t>re_ap11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6711,7 +6711,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rg_ap12</t>
+          <t>re_ap12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6759,7 +6759,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>rg_ap13</t>
+          <t>re_ap13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rg_vi1</t>
+          <t>re_vi1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6965,7 +6965,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rg_vi2</t>
+          <t>re_vi2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -7013,7 +7013,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rg_vi3</t>
+          <t>re_vi3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -7061,7 +7061,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rg_vi4</t>
+          <t>re_vi4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -7109,7 +7109,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rg_vi5</t>
+          <t>re_vi5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rg_vi6</t>
+          <t>re_vi6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7205,7 +7205,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rg_vi7</t>
+          <t>re_vi7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -7253,7 +7253,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>rg_vi8</t>
+          <t>re_vi8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7301,7 +7301,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>rg_vi9</t>
+          <t>re_vi9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7349,7 +7349,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>rg_vi10</t>
+          <t>re_vi10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>rg_vi11</t>
+          <t>re_vi11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7445,7 +7445,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rg_vi12</t>
+          <t>re_vi12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7493,7 +7493,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>rg_vi13</t>
+          <t>re_vi13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7651,7 +7651,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rg_so1</t>
+          <t>re_so1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -7699,7 +7699,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rg_so2</t>
+          <t>re_so2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -7747,7 +7747,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rg_so3</t>
+          <t>re_so3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -7795,7 +7795,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rg_so4</t>
+          <t>re_so4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -7843,7 +7843,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rg_so5</t>
+          <t>re_so5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7891,7 +7891,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rg_so6</t>
+          <t>re_so6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7939,7 +7939,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rg_so7</t>
+          <t>re_so7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">

</xml_diff>